<commit_message>
changed to use sql in calculations
</commit_message>
<xml_diff>
--- a/data/report_template.xlsx
+++ b/data/report_template.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Documents/Python Scripts/DashPlotly/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD096A4-7C31-2D41-AD56-B0873E220A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF742739-17A5-4A42-B99F-9F5E8F7AE682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1600" yWindow="760" windowWidth="29900" windowHeight="19880" activeTab="3" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
+    <workbookView xWindow="1600" yWindow="760" windowWidth="29900" windowHeight="19880" activeTab="2" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
   </bookViews>
   <sheets>
     <sheet name="VARIABLE_NAMES" sheetId="1" r:id="rId1"/>
     <sheet name="FILTERS" sheetId="2" r:id="rId2"/>
-    <sheet name="REPORT_NAME" sheetId="3" r:id="rId3"/>
-    <sheet name="EXAMPLES" sheetId="9" r:id="rId4"/>
+    <sheet name="GUIDE" sheetId="10" r:id="rId3"/>
+    <sheet name="REPORT_NAME" sheetId="3" r:id="rId4"/>
+    <sheet name="EXAMPLES" sheetId="9" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="687">
   <si>
     <t>name</t>
   </si>
@@ -1854,13 +1855,1711 @@
   </si>
   <si>
     <t>ISDG5HDIF</t>
+  </si>
+  <si>
+    <t>FILTERS Sheet — Filling Guide</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Each row in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FILTERS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sheet defines one named filter whose computed value can be placed anywhere in the report via the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>VARIABLE_NAMES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sheet.</t>
+    </r>
+  </si>
+  <si>
+    <t>Column reference</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>✅</t>
+  </si>
+  <si>
+    <t>Unique identifier for this filter. Referenced by the VARIABLE_NAMES sheet. No spaces recommended (use underscores).</t>
+  </si>
+  <si>
+    <t>What computation to perform. See measure types below.</t>
+  </si>
+  <si>
+    <t>✅*</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The column used to group/aggregate (e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>patient_id</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">). For </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>calculated</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> measure, put the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>expression</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> here instead.</t>
+    </r>
+  </si>
+  <si>
+    <t>num_field</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Numeric column to sum (only used by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>sum</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>cohort_sum</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>). Defaults to the system numeric field if blank.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>variable1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> … </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variable9</t>
+    </r>
+  </si>
+  <si>
+    <t>Data columns to filter on. Add pairs left-to-right; stop when no more conditions are needed.</t>
+  </si>
+  <si>
+    <r>
+      <t>value1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> … </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value9</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Accepted value(s) for the matching </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variableN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column.</t>
+    </r>
+  </si>
+  <si>
+    <t>literal_value</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Only for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> measure. The exact text/number to display.</t>
+    </r>
+  </si>
+  <si>
+    <t>numerator_filter</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Only for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>percentage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> measure. The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>filter_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> of the numerator row.</t>
+    </r>
+  </si>
+  <si>
+    <t>denominator_filter</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Only for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>percentage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> measure. The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>filter_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> of the denominator row.</t>
+    </r>
+  </si>
+  <si>
+    <t>Measure types</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Counts rows in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>filtered</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset matching all variable/value pairs.</t>
+    </r>
+  </si>
+  <si>
+    <t>new_clients</t>
+  </si>
+  <si>
+    <t>patient_id</t>
+  </si>
+  <si>
+    <t>enrollment_type</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>nunique</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Same behaviour as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>count</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (counts distinct unique_column entries). Use when you want to be explicit that you are counting unique individuals.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Counts using set logic (each unique_column counted once per matching set of conditions). Uses the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>filtered</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Like </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>count</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> but runs against the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>original (unfiltered)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset. Use for cohort denominators that must not be restricted by the active date/site filter.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Like </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>count_set</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> but against the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>original</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>count_defaulter</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13.5"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>cohort_count_defaulter</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13.5"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>cohort_count_set_defaulter</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Defaulter variants. Behave like their base measure but automatically include the appointment/defaulter-related columns (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>concept_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value_datetime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) in the query. Use for missed-appointment or IIT indicators.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sums the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>num_field</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column for matching rows. Uses the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>filtered</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset.</t>
+    </r>
+  </si>
+  <si>
+    <t>total_cd4</t>
+  </si>
+  <si>
+    <t>cd4_value</t>
+  </si>
+  <si>
+    <t>test_type</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Like </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>sum</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> but against the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>original</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dataset.</t>
+    </r>
+  </si>
+  <si>
+    <t>percentage</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Divides one filter's result by another and multiplies by 100. Result is displayed as e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>87.5%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leave all </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variableN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>valueN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> columns blank. Fill only:</t>
+    </r>
+  </si>
+  <si>
+    <t>vl_suppression_rate</t>
+  </si>
+  <si>
+    <t>vl_suppressed</t>
+  </si>
+  <si>
+    <t>vl_tested</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Both </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>numerator_filter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>denominator_filter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>filter_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> values defined elsewhere in the sheet.</t>
+    </r>
+  </si>
+  <si>
+    <t>literal</t>
+  </si>
+  <si>
+    <t>Outputs a fixed text or number exactly as written. Useful for static labels or target values.</t>
+  </si>
+  <si>
+    <t>target_label</t>
+  </si>
+  <si>
+    <t>Leave all other columns blank.</t>
+  </si>
+  <si>
+    <t>calculated</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Evaluates an arithmetic expression referencing other filters by name. The expression goes in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>unique_column</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column (not </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal_value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write filter names wrapped in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>{}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Standard operators </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are supported.</t>
+    </r>
+  </si>
+  <si>
+    <t>net_new</t>
+  </si>
+  <si>
+    <t>{enrolled} - {transferred_out}</t>
+  </si>
+  <si>
+    <t>ratio_per_100</t>
+  </si>
+  <si>
+    <t>{positive} / {tested} * 100</t>
+  </si>
+  <si>
+    <t>Formatting rules applied automatically:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Expression contains </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → result rounded to max 2 decimal places (trailing zeros removed, e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3.50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">No </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → result is a whole integer, no decimal places</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">All filters referenced in the expression are computed before any </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>calculated</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> filter is evaluated, so the referenced filters may be defined in any order and can belong to different report sections.</t>
+    </r>
+  </si>
+  <si>
+    <t>Filtering values — syntax</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A single </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>valueN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cell can hold one value, a list, or a pipe-separated set:</t>
+    </r>
+  </si>
+  <si>
+    <t>Syntax</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Match exactly </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>Positive</t>
+    </r>
+  </si>
+  <si>
+    <t>Positive|Reactive</t>
+  </si>
+  <si>
+    <t>Match either value (OR logic)</t>
+  </si>
+  <si>
+    <t>[Positive, Reactive]</t>
+  </si>
+  <si>
+    <t>Same — bracket list syntax</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A blank </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>valueN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> means no filtering on that variable (all values accepted).</t>
+    </r>
+  </si>
+  <si>
+    <t>Quick rules</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Every row must have a unique </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>filter_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Duplicate names silently overwrite each other.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>variable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pairs are read left-to-right and stop at the first blank </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variableN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Do not leave gaps in the middle.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">For </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>calculated</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, leave </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>num_field</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal_value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>numerator_filter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>denominator_filter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and all </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> columns blank.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">For </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>percentage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, leave </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>unique_column</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>num_field</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal_value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and all </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>variable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> columns blank.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">For </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, only </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>filter_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>measure</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>literal_value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are needed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>cohort_*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> measures query the full original dataset regardless of the active report date range or site filter. All other measures query the pre-filtered dataset.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1907,6 +3606,51 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1940,7 +3684,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1950,13 +3694,29 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2485,53 +4245,557 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{73ED4B6C-9864-8A41-958D-522FACDCBD08}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576 J2:J1048576 L2:L1048576 N2:N1048576 C2:F1048576" xr:uid="{D1FD860E-88EF-6C46-BE53-7A4DBF0A8B6D}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{73ED4B6C-9864-8A41-958D-522FACDCBD08}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2:B1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D1FD860E-88EF-6C46-BE53-7A4DBF0A8B6D}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E738FA70-C97B-634E-9058-B830F6B3CC9B}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5360F4A-CE4D-034B-AADF-65DBB821B4DC}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F9B71D13-3A6F-D847-92EA-05112148CA16}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{41B61C2E-BD9D-1848-9292-CD17FE55DEB6}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>H2:H1048576 J2:J1048576 L2:L1048576 N2:N1048576</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA03B3C-D6B0-664D-9360-345FA799876A}">
+  <dimension ref="A1:G124"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="68.5" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="64" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="25" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="13" t="s">
+        <v>608</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>609</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>611</v>
+      </c>
+      <c r="C7" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>611</v>
+      </c>
+      <c r="C8" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>614</v>
+      </c>
+      <c r="C9" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>616</v>
+      </c>
+      <c r="B10" t="s">
+        <v>617</v>
+      </c>
+      <c r="C10" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
+        <v>619</v>
+      </c>
+      <c r="B11" t="s">
+        <v>617</v>
+      </c>
+      <c r="C11" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>621</v>
+      </c>
+      <c r="B12" t="s">
+        <v>617</v>
+      </c>
+      <c r="C12" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A13" s="14" t="s">
+        <v>623</v>
+      </c>
+      <c r="B13" t="s">
+        <v>617</v>
+      </c>
+      <c r="C13" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>625</v>
+      </c>
+      <c r="B14" t="s">
+        <v>617</v>
+      </c>
+      <c r="C14" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
+        <v>627</v>
+      </c>
+      <c r="B15" t="s">
+        <v>617</v>
+      </c>
+      <c r="C15" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="25" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="B23" t="s">
+        <v>587</v>
+      </c>
+      <c r="C23" t="s">
+        <v>632</v>
+      </c>
+      <c r="D23" t="s">
+        <v>633</v>
+      </c>
+      <c r="E23" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="35" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="35" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A40" s="15" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="20" x14ac:dyDescent="0.25">
+      <c r="A45" s="15" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="52" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A50" s="15" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A53" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>616</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="B54" t="s">
+        <v>589</v>
+      </c>
+      <c r="C54" t="s">
+        <v>632</v>
+      </c>
+      <c r="D54" t="s">
+        <v>644</v>
+      </c>
+      <c r="E54" t="s">
+        <v>645</v>
+      </c>
+      <c r="F54" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="17" x14ac:dyDescent="0.25">
+      <c r="A62" s="15" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="35" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A67" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>625</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="B68" t="s">
+        <v>647</v>
+      </c>
+      <c r="C68" t="s">
+        <v>651</v>
+      </c>
+      <c r="D68" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="17" x14ac:dyDescent="0.25">
+      <c r="A74" s="15" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A78" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B78" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="9" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B79" t="s">
+        <v>654</v>
+      </c>
+      <c r="C79">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="17" x14ac:dyDescent="0.25">
+      <c r="A85" s="15" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="52" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="36" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A91" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B91" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C91" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+      <c r="A92" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="B92" t="s">
+        <v>658</v>
+      </c>
+      <c r="C92" s="10" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="B93" t="s">
+        <v>658</v>
+      </c>
+      <c r="C93" s="10" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A95" s="13" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="54" x14ac:dyDescent="0.25">
+      <c r="A97" s="1" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A98" s="1" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="69" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="25" x14ac:dyDescent="0.3">
+      <c r="A104" s="12" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="35" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A108" s="13" t="s">
+        <v>671</v>
+      </c>
+      <c r="B108" s="9" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A109" s="14" t="s">
+        <v>673</v>
+      </c>
+      <c r="B109" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A110" s="14" t="s">
+        <v>675</v>
+      </c>
+      <c r="B110" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="17" x14ac:dyDescent="0.25">
+      <c r="A111" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="B111" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" ht="35" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A117" s="12" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" ht="35" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" ht="53" x14ac:dyDescent="0.2">
+      <c r="A120" s="14" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" ht="54" x14ac:dyDescent="0.25">
+      <c r="A121" s="1" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A122" s="1" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" ht="35" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" ht="69" x14ac:dyDescent="0.2">
+      <c r="A124" s="14" t="s">
+        <v>686</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99E53CD3-50A0-1347-AEEF-73E1C95C94BD}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2564,7 +4828,7 @@
       <c r="C2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" t="s">
         <v>604</v>
       </c>
     </row>
@@ -2573,37 +4837,37 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6821880E-E76E-1B42-A3D1-133D5CF5E1BB}">
   <dimension ref="A1:I492"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>585</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>586</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>593</v>
       </c>
     </row>
@@ -2614,13 +4878,13 @@
       <c r="B2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>584</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>584</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>46</v>
       </c>
       <c r="F2" s="4" t="s">
@@ -2646,7 +4910,7 @@
       <c r="C3" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>47</v>
       </c>
       <c r="F3" s="4" t="s">
@@ -2672,13 +4936,13 @@
       <c r="C4" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>48</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>589</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="8" t="s">
         <v>596</v>
       </c>
       <c r="I4" s="4" t="s">
@@ -2695,7 +4959,7 @@
       <c r="C5" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>49</v>
       </c>
       <c r="G5" s="4" t="s">
@@ -2754,7 +5018,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>601</v>
       </c>
       <c r="B9" s="4" t="s">

</xml_diff>